<commit_message>
EPBDS-14557 addressed review comments
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.test/test-resources/functionality/EPBDS-14557_Vocabulary_Validation.xlsx
+++ b/STUDIO/org.openl.rules.test/test-resources/functionality/EPBDS-14557_Vocabulary_Validation.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdeshmane/Downloads/"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="63">
   <si>
     <t>Datatype Gender &lt;String&gt;</t>
   </si>
@@ -164,12 +164,58 @@
   </si>
   <si>
     <t>= SomeMethod (new String[]{"Test12"}, 10)</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test1","F1", 100)</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test3","F3",5)</t>
+  </si>
+  <si>
+    <t>= SomeMethod(new String[] {"Test14", "test"},new Integer[]{10, 20})</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test4","F4",new Integer[] {125, 200, 225})</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test2","Female", 2)</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test3","F3",3)</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test4","F4",new Integer[] {124, 200, 224})</t>
+  </si>
+  <si>
+    <t>= GenderFactor ("test5", new String[]{"F5","M5"}, new Integer[] {135, 300, 245})</t>
+  </si>
+  <si>
+    <t>= SomeMethod ("Test6", 10)</t>
+  </si>
+  <si>
+    <t>= SomeMethod ("Test6", 6)</t>
+  </si>
+  <si>
+    <t>= SomeMethod (new String[]{"Test7"}, 10)</t>
+  </si>
+  <si>
+    <t>= SomeMethod (new String[]{"Test8"}, new Integer[]{10, 20})</t>
+  </si>
+  <si>
+    <t>= SomeMethod (new String[]{"Test8"}, new Integer[]{10, 28})</t>
+  </si>
+  <si>
+    <t>= SomeMethod(new String[] {"Test19", "test29"},new Integer[]{10, 29})</t>
+  </si>
+  <si>
+    <t>= GenderFactor(new String[] {"test6"}, new String[]{"F6", "M6"}, new Integer[] {100, 136, 356})</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="9">
     <font>
       <sz val="10"/>
@@ -374,7 +420,7 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -790,18 +836,18 @@
   <dimension ref="B3:E42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="2.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="31.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="41.83203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.1640625" style="1"/>
+    <col min="1" max="1" customWidth="true" style="1" width="2.83203125"/>
+    <col min="2" max="2" customWidth="true" style="1" width="19.33203125"/>
+    <col min="3" max="3" customWidth="true" style="1" width="31.6640625"/>
+    <col min="4" max="4" customWidth="true" style="1" width="41.83203125"/>
+    <col min="5" max="5" customWidth="true" style="1" width="24.33203125"/>
+    <col min="6" max="6" customWidth="true" style="1" width="25.83203125"/>
+    <col min="7" max="7" customWidth="true" style="1" width="11.5"/>
+    <col min="8" max="8" customWidth="true" style="1" width="12.83203125"/>
+    <col min="9" max="9" customWidth="true" style="1" width="14.33203125"/>
+    <col min="10" max="10" customWidth="true" style="1" width="12.83203125"/>
+    <col min="11" max="11" customWidth="true" style="1" width="13.0"/>
+    <col min="12" max="16384" style="1" width="9.1640625"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:2" ht="14" thickBot="1"/>
@@ -947,7 +993,7 @@
         <v>12</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>10</v>
@@ -958,7 +1004,7 @@
         <v>19</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D30" s="9"/>
     </row>
@@ -967,7 +1013,7 @@
         <v>21</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="D31" s="9"/>
     </row>
@@ -976,7 +1022,7 @@
         <v>23</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="D32" s="9"/>
     </row>
@@ -985,7 +1031,7 @@
         <v>24</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="D33" s="9"/>
     </row>
@@ -994,7 +1040,7 @@
         <v>25</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="D34" s="9"/>
     </row>
@@ -1003,7 +1049,7 @@
         <v>26</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="D35" s="9"/>
     </row>
@@ -1012,7 +1058,7 @@
         <v>27</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="D36" s="9"/>
     </row>
@@ -1021,7 +1067,7 @@
         <v>28</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="D37" s="9"/>
     </row>
@@ -1029,47 +1075,15 @@
       <c r="B38" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C38" s="11" t="s">
-        <v>34</v>
+      <c r="C38" t="s" s="11">
+        <v>61</v>
       </c>
       <c r="D38" s="9"/>
     </row>
-    <row r="39" spans="2:4">
-      <c r="B39" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D39" s="9"/>
-    </row>
-    <row r="40" spans="2:4">
-      <c r="B40" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="D40" s="9"/>
-    </row>
-    <row r="41" spans="2:4">
-      <c r="B41" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="D41" s="9"/>
-    </row>
-    <row r="42" spans="2:4">
-      <c r="B42" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="D42" s="9"/>
-    </row>
+    <row r="39" spans="2:4"/>
+    <row r="40" spans="2:4"/>
+    <row r="41" spans="2:4"/>
+    <row r="42" spans="2:4"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B22:D22"/>

</xml_diff>

<commit_message>
EPBDS-14557 var args parameter scenario
</commit_message>
<xml_diff>
--- a/STUDIO/org.openl.rules.test/test-resources/functionality/EPBDS-14557_Vocabulary_Validation.xlsx
+++ b/STUDIO/org.openl.rules.test/test-resources/functionality/EPBDS-14557_Vocabulary_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdeshmane/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42627A1D-4FC6-1340-BEB8-2BA59E1640B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C76512-31BE-E748-8AA7-4C78814326F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29920" windowHeight="17280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="72">
   <si>
     <t>Datatype Gender &lt;String&gt;</t>
   </si>
@@ -218,9 +218,6 @@
     <t>error</t>
   </si>
   <si>
-    <t>Spreadsheet SpreadsheetResult check(County county)</t>
-  </si>
-  <si>
     <t>Result</t>
   </si>
   <si>
@@ -228,6 +225,30 @@
   </si>
   <si>
     <t>= country</t>
+  </si>
+  <si>
+    <t>SimpleRules Double SomeMethod1(String[] test, Integer no)</t>
+  </si>
+  <si>
+    <t>Check19</t>
+  </si>
+  <si>
+    <t>= SomeMethod1(10, "Test1", "Test2")</t>
+  </si>
+  <si>
+    <t>SimpleRules Double SomeMethod1(Integer no, String[] test)</t>
+  </si>
+  <si>
+    <t>= SomeMethod1(10, "Test1")</t>
+  </si>
+  <si>
+    <t>= SomeMethod1(10, "Test1", 0)</t>
+  </si>
+  <si>
+    <t>= SomeMethod1(10, "Test199", "test19')</t>
+  </si>
+  <si>
+    <t>= SomeMethod1(10, "Test199", "test19")</t>
   </si>
 </sst>
 </file>
@@ -283,7 +304,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -311,27 +332,13 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="solid"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -458,54 +465,6 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thick"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <bottom style="thick"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <bottom style="thick"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thick"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thick">
-        <color indexed="0"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="0"/>
-      </left>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thick">
-        <color indexed="0"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="0"/>
-      </left>
-      <right style="thin">
-        <color indexed="0"/>
-      </right>
-      <top style="thin"/>
-      <bottom style="thick">
-        <color indexed="0"/>
-      </bottom>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="0"/>
       </left>
@@ -518,6 +477,7 @@
       <bottom style="thick">
         <color indexed="0"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -561,6 +521,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -569,10 +532,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="18" xfId="0" applyAlignment="true" applyBorder="true" applyNumberFormat="true" applyFill="true" applyFont="true" quotePrefix="false">
-      <alignment horizontal="left" vertical="bottom" indent="0" textRotation="0" wrapText="false" shrinkToFit="false"/>
-      <protection hidden="false" locked="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,7 +898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B4:E51"/>
+  <dimension ref="B4:E60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="2.83203125"/>
@@ -1007,12 +966,12 @@
       </c>
     </row>
     <row r="17" spans="2:5">
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="3" t="s">
@@ -1058,11 +1017,11 @@
     </row>
     <row r="21" spans="2:5" ht="14" thickTop="1"/>
     <row r="22" spans="2:5">
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="3" t="s">
@@ -1088,11 +1047,11 @@
     </row>
     <row r="25" spans="2:5" ht="14" thickTop="1"/>
     <row r="27" spans="2:5">
-      <c r="B27" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
+      <c r="B27" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
     </row>
     <row r="28" spans="2:5">
       <c r="B28" s="3" t="s">
@@ -1104,19 +1063,19 @@
     </row>
     <row r="29" spans="2:5" ht="14" thickBot="1">
       <c r="B29" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>64</v>
+        <v>61</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="14" thickTop="1"/>
     <row r="32" spans="2:5">
-      <c r="B32" s="16" t="s">
+      <c r="B32" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
     </row>
     <row r="33" spans="2:5" ht="14" thickBot="1">
       <c r="B33" s="3" t="s">
@@ -1310,12 +1269,54 @@
         <v>44</v>
       </c>
     </row>
+    <row r="52">
+      <c r="B52" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" ht="14" thickBot="1">
+      <c r="B59" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="2:4" ht="14" thickTop="1"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B57:D57"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>